<commit_message>
Test end-to-end automation pipeline
</commit_message>
<xml_diff>
--- a/KAHF_Consolidated_Fund_Model  Updated.xlsx
+++ b/KAHF_Consolidated_Fund_Model  Updated.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://konigsteincapital.sharepoint.com/sites/kc-group/Shared Documents/General/Portfolio/KAHF/Fund Model/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://konigsteincapital-my.sharepoint.com/personal/wayne_konigsteincapital_com/Documents/Project Images/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1499" documentId="8_{9150A69C-E6E4-4446-B489-F85005C0890C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7AF972A3-E2A5-4A81-8F8D-1AC8E48F3715}"/>
+  <xr:revisionPtr revIDLastSave="1500" documentId="8_{9150A69C-E6E4-4446-B489-F85005C0890C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{379ACD62-8115-43E3-9302-EB0857A0BBD6}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-4200" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Dashboard &amp; Jun-26" sheetId="1" r:id="rId1"/>
@@ -182,7 +182,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -1622,8 +1622,8 @@
     <numFmt numFmtId="172" formatCode="#,##0.00;&quot;(&quot;#,##0.00&quot;)&quot;;&quot;-&quot;"/>
     <numFmt numFmtId="173" formatCode="dd&quot; &quot;mmm&quot; &quot;yyyy"/>
     <numFmt numFmtId="174" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="178" formatCode="0.000%"/>
-    <numFmt numFmtId="179" formatCode="0.000000%"/>
+    <numFmt numFmtId="175" formatCode="0.000%"/>
+    <numFmt numFmtId="176" formatCode="0.000000%"/>
   </numFmts>
   <fonts count="44" x14ac:knownFonts="1">
     <font>
@@ -1877,6 +1877,7 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -2357,21 +2358,21 @@
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="38" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="178" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="39" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="175" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="40" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="179" fontId="41" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="176" fontId="41" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="41" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="39" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -2401,46 +2402,8 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
-    </dxf>
-    <dxf>
-      <font>
         <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="22" formatCode="mmm\-yy"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
+        <i/>
         <strike val="0"/>
         <condense val="0"/>
         <extend val="0"/>
@@ -2458,7 +2421,7 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
+        <b/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -2468,64 +2431,7 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="168" formatCode="d\-mmm\-yy"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
+        <color rgb="FF000000"/>
         <name val="Arial"/>
         <family val="2"/>
         <scheme val="none"/>
@@ -2623,6 +2529,25 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="22" formatCode="mmm\-yy"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
       <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
     </dxf>
     <dxf>
@@ -2638,6 +2563,63 @@
         <vertAlign val="baseline"/>
         <sz val="10"/>
         <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
         <name val="Arial"/>
         <family val="2"/>
         <scheme val="none"/>
@@ -2698,6 +2680,25 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="168" formatCode="d\-mmm\-yy"/>
     </dxf>
     <dxf>
       <font>
@@ -4603,10 +4604,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2745D919-B1B2-4FDF-B950-9727D6F2E18A}" name="Table1" displayName="Table1" ref="A4:I125" totalsRowCount="1" headerRowDxfId="18">
   <autoFilter ref="A4:I124" xr:uid="{2745D919-B1B2-4FDF-B950-9727D6F2E18A}"/>
@@ -4614,23 +4611,23 @@
     <sortCondition ref="A5:A124"/>
   </sortState>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{1CC3A698-EDA3-4671-B907-22AA32065BD2}" name="Date" dataDxfId="17" totalsRowDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{A235E874-F2C8-4F6D-B44C-A2C2D5DC77F3}" name="Project" dataDxfId="16" totalsRowDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{BD5A1FAA-F155-4713-8E06-0C317B10A3D0}" name="Amount (N$)" dataDxfId="14" totalsRowDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{8BA57056-D260-4F3C-8D82-76DBDF26EFF1}" name="Drawdown (N$)" totalsRowFunction="sum" dataDxfId="13" totalsRowDxfId="4" dataCellStyle="Comma">
+    <tableColumn id="1" xr3:uid="{1CC3A698-EDA3-4671-B907-22AA32065BD2}" name="Date" dataDxfId="17" totalsRowDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{A235E874-F2C8-4F6D-B44C-A2C2D5DC77F3}" name="Project" dataDxfId="15" totalsRowDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{BD5A1FAA-F155-4713-8E06-0C317B10A3D0}" name="Amount (N$)" dataDxfId="13" totalsRowDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{8BA57056-D260-4F3C-8D82-76DBDF26EFF1}" name="Drawdown (N$)" totalsRowFunction="sum" dataDxfId="11" totalsRowDxfId="10" dataCellStyle="Comma">
       <calculatedColumnFormula>IF(C5&lt;0,C5,0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{E86CBD51-5855-4402-8499-73E7044F5C14}" name="Distribution (N$)" totalsRowFunction="sum" dataDxfId="12" totalsRowDxfId="3">
+    <tableColumn id="5" xr3:uid="{E86CBD51-5855-4402-8499-73E7044F5C14}" name="Distribution (N$)" totalsRowFunction="sum" dataDxfId="9" totalsRowDxfId="8">
       <calculatedColumnFormula>IF(C5&gt;0,C5,0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{78EFF85F-09AE-43AA-B662-93DD05540FD6}" name="Month key" dataDxfId="11" totalsRowDxfId="2">
+    <tableColumn id="6" xr3:uid="{78EFF85F-09AE-43AA-B662-93DD05540FD6}" name="Month key" dataDxfId="7" totalsRowDxfId="6">
       <calculatedColumnFormula>DATE(YEAR(A5),MONTH(A5),1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{A9E613AA-2076-45AD-A76E-C933EA14771C}" name="Source workbook / tab" dataDxfId="10" totalsRowDxfId="9"/>
-    <tableColumn id="8" xr3:uid="{B74CB5D9-AC93-43D8-BA31-8C4A80990DD3}" name="Management Account (N$)" totalsRowFunction="sum" dataDxfId="8" totalsRowDxfId="1">
+    <tableColumn id="7" xr3:uid="{A9E613AA-2076-45AD-A76E-C933EA14771C}" name="Source workbook / tab" dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{B74CB5D9-AC93-43D8-BA31-8C4A80990DD3}" name="Management Account (N$)" totalsRowFunction="sum" dataDxfId="3" totalsRowDxfId="2">
       <calculatedColumnFormula>IFERROR(_xlfn.XLOOKUP($A5,$M$5:$M$94,$O$5:$O$94),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{732F6E87-E85F-47AD-A11A-46CD028811CC}" name="Permitted Expenses (N$)" totalsRowFunction="sum" dataDxfId="7" totalsRowDxfId="0">
+    <tableColumn id="9" xr3:uid="{732F6E87-E85F-47AD-A11A-46CD028811CC}" name="Permitted Expenses (N$)" totalsRowFunction="sum" dataDxfId="1" totalsRowDxfId="0">
       <calculatedColumnFormula>IFERROR(_xlfn.XLOOKUP($A5,$M$5:$M$94,$P$5:$P$94),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5495,7 +5492,7 @@
         <v>0.80679453239954835</v>
       </c>
       <c r="M5" s="16">
-        <v>5.4100000000000002E-2</v>
+        <v>8.7400000000000005E-2</v>
       </c>
       <c r="N5" s="17" t="s">
         <v>73</v>
@@ -6158,7 +6155,7 @@
       </c>
       <c r="M19" s="72">
         <f>(M5+M18+M17+M16+M15+M14+M13+M11+M10+M9-M8+M6+M7+M20)/13</f>
-        <v>0.18674615384615384</v>
+        <v>0.18930769230769234</v>
       </c>
       <c r="N19" s="20"/>
     </row>
@@ -6240,10 +6237,10 @@
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="O30" s="161" t="s">
+      <c r="O30" s="172" t="s">
         <v>321</v>
       </c>
-      <c r="P30" s="161"/>
+      <c r="P30" s="172"/>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.3">
       <c r="P31" t="s">
@@ -12180,12 +12177,12 @@
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="M3" s="166" t="s">
+      <c r="M3" s="173" t="s">
         <v>456</v>
       </c>
-      <c r="N3" s="166"/>
-      <c r="O3" s="166"/>
-      <c r="P3" s="166"/>
+      <c r="N3" s="173"/>
+      <c r="O3" s="173"/>
+      <c r="P3" s="173"/>
     </row>
     <row r="4" spans="1:16" ht="42" x14ac:dyDescent="0.3">
       <c r="A4" s="35" t="s">
@@ -13734,7 +13731,7 @@
         <v>0</v>
       </c>
       <c r="I37" s="39">
-        <f t="shared" ref="I37:I68" si="8">IFERROR(_xlfn.XLOOKUP($A37,$M$5:$M$94,$P$5:$P$94),0)</f>
+        <f t="shared" ref="I37:I67" si="8">IFERROR(_xlfn.XLOOKUP($A37,$M$5:$M$94,$P$5:$P$94),0)</f>
         <v>0</v>
       </c>
       <c r="M37" s="157">
@@ -15242,7 +15239,7 @@
         <v>0</v>
       </c>
       <c r="I70" s="39">
-        <f t="shared" ref="I69:I100" si="13">IFERROR(_xlfn.XLOOKUP($A70,$M$5:$M$94,$P$5:$P$94),0)</f>
+        <f t="shared" ref="I70:I100" si="13">IFERROR(_xlfn.XLOOKUP($A70,$M$5:$M$94,$P$5:$P$94),0)</f>
         <v>0</v>
       </c>
       <c r="M70" s="157">
@@ -16581,7 +16578,7 @@
         <v>-4700000</v>
       </c>
       <c r="D101" s="39">
-        <f t="shared" ref="D101:D132" si="14">IF(C101&lt;0,C101,0)</f>
+        <f t="shared" ref="D101:D124" si="14">IF(C101&lt;0,C101,0)</f>
         <v>-4700000</v>
       </c>
       <c r="E101" s="39">
@@ -17710,7 +17707,7 @@
       <c r="A1" s="44" t="s">
         <v>182</v>
       </c>
-      <c r="J1" s="168" t="s">
+      <c r="J1" s="165" t="s">
         <v>464</v>
       </c>
     </row>
@@ -17718,31 +17715,31 @@
       <c r="A2" s="45" t="s">
         <v>196</v>
       </c>
-      <c r="J2" s="170" t="s">
+      <c r="J2" s="167" t="s">
         <v>458</v>
       </c>
-      <c r="K2" s="170" t="s">
+      <c r="K2" s="167" t="s">
         <v>459</v>
       </c>
-      <c r="L2" s="170" t="s">
+      <c r="L2" s="167" t="s">
         <v>460</v>
       </c>
-      <c r="M2" s="170" t="s">
+      <c r="M2" s="167" t="s">
         <v>465</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="J3" s="171">
+      <c r="J3" s="168">
         <v>-0.5</v>
       </c>
-      <c r="K3" s="171">
+      <c r="K3" s="168">
         <v>0.5</v>
       </c>
-      <c r="L3" s="172">
+      <c r="L3" s="169">
         <f>(J3+K3)/2</f>
         <v>0</v>
       </c>
-      <c r="M3" s="173" cm="1">
+      <c r="M3" s="170" cm="1">
         <f t="array" ref="M3">SUMPRODUCT($H$6:$H$127,(1+L3)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>36389837.315467715</v>
       </c>
@@ -17752,22 +17749,22 @@
         <v>183</v>
       </c>
       <c r="B4" s="47"/>
-      <c r="C4" s="162"/>
-      <c r="D4" s="162"/>
-      <c r="E4" s="162"/>
-      <c r="J4" s="169">
+      <c r="C4" s="171"/>
+      <c r="D4" s="171"/>
+      <c r="E4" s="171"/>
+      <c r="J4" s="166">
         <f>IF(M3&gt;0,L3,J3)</f>
         <v>0</v>
       </c>
-      <c r="K4" s="169">
+      <c r="K4" s="166">
         <f>IF(M3&gt;0,K3,L3)</f>
         <v>0.5</v>
       </c>
-      <c r="L4" s="172">
+      <c r="L4" s="169">
         <f>(J4+K4)/2</f>
         <v>0.25</v>
       </c>
-      <c r="M4" s="173" cm="1">
+      <c r="M4" s="170" cm="1">
         <f t="array" ref="M4">SUMPRODUCT($H$6:$H$127,(1+L4)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>-29816208.091465957</v>
       </c>
@@ -17794,19 +17791,19 @@
       <c r="H5" s="49" t="s">
         <v>461</v>
       </c>
-      <c r="J5" s="169">
+      <c r="J5" s="166">
         <f t="shared" ref="J5:J42" si="0">IF(M4&gt;0,L4,J4)</f>
         <v>0</v>
       </c>
-      <c r="K5" s="169">
+      <c r="K5" s="166">
         <f t="shared" ref="K5:K42" si="1">IF(M4&gt;0,K4,L4)</f>
         <v>0.25</v>
       </c>
-      <c r="L5" s="172">
+      <c r="L5" s="169">
         <f t="shared" ref="L5:L42" si="2">(J5+K5)/2</f>
         <v>0.125</v>
       </c>
-      <c r="M5" s="173" cm="1">
+      <c r="M5" s="170" cm="1">
         <f t="array" ref="M5">SUMPRODUCT($H$6:$H$127,(1+L5)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>-13696417.962732753</v>
       </c>
@@ -17832,7 +17829,7 @@
         <f t="shared" ref="E6:E37" si="4">C6-D6</f>
         <v>0</v>
       </c>
-      <c r="G6" s="167">
+      <c r="G6" s="164">
         <f>-IF(COUNTIF($A$6:A6,A6)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A6)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A6),0)</f>
         <v>-1533615</v>
       </c>
@@ -17840,19 +17837,19 @@
         <f>C6+G6</f>
         <v>-1533615</v>
       </c>
-      <c r="J6" s="169">
+      <c r="J6" s="166">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K6" s="169">
+      <c r="K6" s="166">
         <f t="shared" si="1"/>
         <v>0.125</v>
       </c>
-      <c r="L6" s="172">
+      <c r="L6" s="169">
         <f t="shared" si="2"/>
         <v>6.25E-2</v>
       </c>
-      <c r="M6" s="173" cm="1">
+      <c r="M6" s="170" cm="1">
         <f t="array" ref="M6">SUMPRODUCT($H$6:$H$127,(1+L6)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>3985327.5389926112</v>
       </c>
@@ -17878,7 +17875,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G7" s="167">
+      <c r="G7" s="164">
         <f>-IF(COUNTIF($A$6:A7,A7)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A7)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A7),0)</f>
         <v>0</v>
       </c>
@@ -17886,19 +17883,19 @@
         <f>C7+G7-D7</f>
         <v>0</v>
       </c>
-      <c r="J7" s="169">
+      <c r="J7" s="166">
         <f t="shared" si="0"/>
         <v>6.25E-2</v>
       </c>
-      <c r="K7" s="169">
+      <c r="K7" s="166">
         <f t="shared" si="1"/>
         <v>0.125</v>
       </c>
-      <c r="L7" s="172">
+      <c r="L7" s="169">
         <f t="shared" si="2"/>
         <v>9.375E-2</v>
       </c>
-      <c r="M7" s="173" cm="1">
+      <c r="M7" s="170" cm="1">
         <f t="array" ref="M7">SUMPRODUCT($H$6:$H$127,(1+L7)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>-6131875.6230139164</v>
       </c>
@@ -17924,7 +17921,7 @@
         <f t="shared" si="4"/>
         <v>-2200000</v>
       </c>
-      <c r="G8" s="167">
+      <c r="G8" s="164">
         <f>-IF(COUNTIF($A$6:A8,A8)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A8)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A8),0)</f>
         <v>0</v>
       </c>
@@ -17932,19 +17929,19 @@
         <f t="shared" ref="H8:H71" si="5">C8+G8-D8</f>
         <v>-2200000</v>
       </c>
-      <c r="J8" s="169">
+      <c r="J8" s="166">
         <f t="shared" si="0"/>
         <v>6.25E-2</v>
       </c>
-      <c r="K8" s="169">
+      <c r="K8" s="166">
         <f t="shared" si="1"/>
         <v>9.375E-2</v>
       </c>
-      <c r="L8" s="172">
+      <c r="L8" s="169">
         <f t="shared" si="2"/>
         <v>7.8125E-2</v>
       </c>
-      <c r="M8" s="173" cm="1">
+      <c r="M8" s="170" cm="1">
         <f t="array" ref="M8">SUMPRODUCT($H$6:$H$127,(1+L8)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>-1447160.2807470015</v>
       </c>
@@ -17970,7 +17967,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G9" s="167">
+      <c r="G9" s="164">
         <f>-IF(COUNTIF($A$6:A9,A9)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A9)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A9),0)</f>
         <v>-1128906.25</v>
       </c>
@@ -17978,19 +17975,19 @@
         <f t="shared" si="5"/>
         <v>-1128906.25</v>
       </c>
-      <c r="J9" s="169">
+      <c r="J9" s="166">
         <f t="shared" si="0"/>
         <v>6.25E-2</v>
       </c>
-      <c r="K9" s="169">
+      <c r="K9" s="166">
         <f t="shared" si="1"/>
         <v>7.8125E-2</v>
       </c>
-      <c r="L9" s="172">
+      <c r="L9" s="169">
         <f t="shared" si="2"/>
         <v>7.03125E-2</v>
       </c>
-      <c r="M9" s="173" cm="1">
+      <c r="M9" s="170" cm="1">
         <f t="array" ref="M9">SUMPRODUCT($H$6:$H$127,(1+L9)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>1167629.9957888154</v>
       </c>
@@ -18016,7 +18013,7 @@
         <f t="shared" si="4"/>
         <v>-22000000</v>
       </c>
-      <c r="G10" s="167">
+      <c r="G10" s="164">
         <f>-IF(COUNTIF($A$6:A10,A10)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A10)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A10),0)</f>
         <v>0</v>
       </c>
@@ -18024,19 +18021,19 @@
         <f t="shared" si="5"/>
         <v>-22000000</v>
       </c>
-      <c r="J10" s="169">
+      <c r="J10" s="166">
         <f t="shared" si="0"/>
         <v>7.03125E-2</v>
       </c>
-      <c r="K10" s="169">
+      <c r="K10" s="166">
         <f t="shared" si="1"/>
         <v>7.8125E-2</v>
       </c>
-      <c r="L10" s="172">
+      <c r="L10" s="169">
         <f t="shared" si="2"/>
         <v>7.421875E-2</v>
       </c>
-      <c r="M10" s="173" cm="1">
+      <c r="M10" s="170" cm="1">
         <f t="array" ref="M10">SUMPRODUCT($H$6:$H$127,(1+L10)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>-164073.75184177514</v>
       </c>
@@ -18062,7 +18059,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G11" s="167">
+      <c r="G11" s="164">
         <f>-IF(COUNTIF($A$6:A11,A11)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A11)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A11),0)</f>
         <v>-1108906.25</v>
       </c>
@@ -18070,19 +18067,19 @@
         <f t="shared" si="5"/>
         <v>-1108906.25</v>
       </c>
-      <c r="J11" s="169">
+      <c r="J11" s="166">
         <f t="shared" si="0"/>
         <v>7.03125E-2</v>
       </c>
-      <c r="K11" s="169">
+      <c r="K11" s="166">
         <f t="shared" si="1"/>
         <v>7.421875E-2</v>
       </c>
-      <c r="L11" s="172">
+      <c r="L11" s="169">
         <f t="shared" si="2"/>
         <v>7.2265625E-2</v>
       </c>
-      <c r="M11" s="173" cm="1">
+      <c r="M11" s="170" cm="1">
         <f t="array" ref="M11">SUMPRODUCT($H$6:$H$127,(1+L11)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>495572.87771679601</v>
       </c>
@@ -18108,7 +18105,7 @@
         <f t="shared" si="4"/>
         <v>-10000000</v>
       </c>
-      <c r="G12" s="167">
+      <c r="G12" s="164">
         <f>-IF(COUNTIF($A$6:A12,A12)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A12)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A12),0)</f>
         <v>0</v>
       </c>
@@ -18116,19 +18113,19 @@
         <f t="shared" si="5"/>
         <v>-10000000</v>
       </c>
-      <c r="J12" s="169">
+      <c r="J12" s="166">
         <f t="shared" si="0"/>
         <v>7.2265625E-2</v>
       </c>
-      <c r="K12" s="169">
+      <c r="K12" s="166">
         <f t="shared" si="1"/>
         <v>7.421875E-2</v>
       </c>
-      <c r="L12" s="172">
+      <c r="L12" s="169">
         <f t="shared" si="2"/>
         <v>7.32421875E-2</v>
       </c>
-      <c r="M12" s="173" cm="1">
+      <c r="M12" s="170" cm="1">
         <f t="array" ref="M12">SUMPRODUCT($H$6:$H$127,(1+L12)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>164214.49192865472</v>
       </c>
@@ -18154,7 +18151,7 @@
         <f t="shared" si="4"/>
         <v>-700000</v>
       </c>
-      <c r="G13" s="167">
+      <c r="G13" s="164">
         <f>-IF(COUNTIF($A$6:A13,A13)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A13)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A13),0)</f>
         <v>-1208740.25</v>
       </c>
@@ -18162,19 +18159,19 @@
         <f t="shared" si="5"/>
         <v>-1908740.25</v>
       </c>
-      <c r="J13" s="169">
+      <c r="J13" s="166">
         <f t="shared" si="0"/>
         <v>7.32421875E-2</v>
       </c>
-      <c r="K13" s="169">
+      <c r="K13" s="166">
         <f t="shared" si="1"/>
         <v>7.421875E-2</v>
       </c>
-      <c r="L13" s="172">
+      <c r="L13" s="169">
         <f t="shared" si="2"/>
         <v>7.373046875E-2</v>
       </c>
-      <c r="M13" s="173" cm="1">
+      <c r="M13" s="170" cm="1">
         <f t="array" ref="M13">SUMPRODUCT($H$6:$H$127,(1+L13)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>-311.38792144926265</v>
       </c>
@@ -18200,7 +18197,7 @@
         <f t="shared" si="4"/>
         <v>-4300000</v>
       </c>
-      <c r="G14" s="167">
+      <c r="G14" s="164">
         <f>-IF(COUNTIF($A$6:A14,A14)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A14)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A14),0)</f>
         <v>0</v>
       </c>
@@ -18208,19 +18205,19 @@
         <f t="shared" si="5"/>
         <v>-4300000</v>
       </c>
-      <c r="J14" s="169">
+      <c r="J14" s="166">
         <f t="shared" si="0"/>
         <v>7.32421875E-2</v>
       </c>
-      <c r="K14" s="169">
+      <c r="K14" s="166">
         <f t="shared" si="1"/>
         <v>7.373046875E-2</v>
       </c>
-      <c r="L14" s="172">
+      <c r="L14" s="169">
         <f t="shared" si="2"/>
         <v>7.3486328125E-2</v>
       </c>
-      <c r="M14" s="173" cm="1">
+      <c r="M14" s="170" cm="1">
         <f t="array" ref="M14">SUMPRODUCT($H$6:$H$127,(1+L14)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>81855.86218445329</v>
       </c>
@@ -18246,7 +18243,7 @@
         <f t="shared" si="4"/>
         <v>-6000000</v>
       </c>
-      <c r="G15" s="167">
+      <c r="G15" s="164">
         <f>-IF(COUNTIF($A$6:A15,A15)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A15)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A15),0)</f>
         <v>0</v>
       </c>
@@ -18254,19 +18251,19 @@
         <f t="shared" si="5"/>
         <v>-6000000</v>
       </c>
-      <c r="J15" s="169">
+      <c r="J15" s="166">
         <f t="shared" si="0"/>
         <v>7.3486328125E-2</v>
       </c>
-      <c r="K15" s="169">
+      <c r="K15" s="166">
         <f t="shared" si="1"/>
         <v>7.373046875E-2</v>
       </c>
-      <c r="L15" s="172">
+      <c r="L15" s="169">
         <f t="shared" si="2"/>
         <v>7.36083984375E-2</v>
       </c>
-      <c r="M15" s="173" cm="1">
+      <c r="M15" s="170" cm="1">
         <f t="array" ref="M15">SUMPRODUCT($H$6:$H$127,(1+L15)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>40748.346023485996</v>
       </c>
@@ -18292,7 +18289,7 @@
         <f t="shared" si="4"/>
         <v>-5000000</v>
       </c>
-      <c r="G16" s="167">
+      <c r="G16" s="164">
         <f>-IF(COUNTIF($A$6:A16,A16)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A16)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A16),0)</f>
         <v>0</v>
       </c>
@@ -18300,19 +18297,19 @@
         <f t="shared" si="5"/>
         <v>-5000000</v>
       </c>
-      <c r="J16" s="169">
+      <c r="J16" s="166">
         <f t="shared" si="0"/>
         <v>7.36083984375E-2</v>
       </c>
-      <c r="K16" s="169">
+      <c r="K16" s="166">
         <f t="shared" si="1"/>
         <v>7.373046875E-2</v>
       </c>
-      <c r="L16" s="172">
+      <c r="L16" s="169">
         <f t="shared" si="2"/>
         <v>7.366943359375E-2</v>
       </c>
-      <c r="M16" s="173" cm="1">
+      <c r="M16" s="170" cm="1">
         <f t="array" ref="M16">SUMPRODUCT($H$6:$H$127,(1+L16)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>20212.510187430773</v>
       </c>
@@ -18338,7 +18335,7 @@
         <f t="shared" si="4"/>
         <v>1302000</v>
       </c>
-      <c r="G17" s="167">
+      <c r="G17" s="164">
         <f>-IF(COUNTIF($A$6:A17,A17)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A17)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A17),0)</f>
         <v>0</v>
       </c>
@@ -18346,19 +18343,19 @@
         <f t="shared" si="5"/>
         <v>1302000</v>
       </c>
-      <c r="J17" s="169">
+      <c r="J17" s="166">
         <f t="shared" si="0"/>
         <v>7.366943359375E-2</v>
       </c>
-      <c r="K17" s="169">
+      <c r="K17" s="166">
         <f t="shared" si="1"/>
         <v>7.373046875E-2</v>
       </c>
-      <c r="L17" s="172">
+      <c r="L17" s="169">
         <f t="shared" si="2"/>
         <v>7.3699951171875E-2</v>
       </c>
-      <c r="M17" s="173" cm="1">
+      <c r="M17" s="170" cm="1">
         <f t="array" ref="M17">SUMPRODUCT($H$6:$H$127,(1+L17)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>9949.0694060004316</v>
       </c>
@@ -18384,7 +18381,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G18" s="167">
+      <c r="G18" s="164">
         <f>-IF(COUNTIF($A$6:A18,A18)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A18)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A18),0)</f>
         <v>-1088906.25</v>
       </c>
@@ -18392,19 +18389,19 @@
         <f t="shared" si="5"/>
         <v>-1088906.25</v>
       </c>
-      <c r="J18" s="169">
+      <c r="J18" s="166">
         <f t="shared" si="0"/>
         <v>7.3699951171875E-2</v>
       </c>
-      <c r="K18" s="169">
+      <c r="K18" s="166">
         <f t="shared" si="1"/>
         <v>7.373046875E-2</v>
       </c>
-      <c r="L18" s="172">
+      <c r="L18" s="169">
         <f t="shared" si="2"/>
         <v>7.37152099609375E-2</v>
       </c>
-      <c r="M18" s="173" cm="1">
+      <c r="M18" s="170" cm="1">
         <f t="array" ref="M18">SUMPRODUCT($H$6:$H$127,(1+L18)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>4818.4678716314957</v>
       </c>
@@ -18430,7 +18427,7 @@
         <f t="shared" si="4"/>
         <v>-1000000</v>
       </c>
-      <c r="G19" s="167">
+      <c r="G19" s="164">
         <f>-IF(COUNTIF($A$6:A19,A19)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A19)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A19),0)</f>
         <v>0</v>
       </c>
@@ -18438,19 +18435,19 @@
         <f t="shared" si="5"/>
         <v>-1000000</v>
       </c>
-      <c r="J19" s="169">
+      <c r="J19" s="166">
         <f t="shared" si="0"/>
         <v>7.37152099609375E-2</v>
       </c>
-      <c r="K19" s="169">
+      <c r="K19" s="166">
         <f t="shared" si="1"/>
         <v>7.373046875E-2</v>
       </c>
-      <c r="L19" s="172">
+      <c r="L19" s="169">
         <f t="shared" si="2"/>
         <v>7.372283935546875E-2</v>
       </c>
-      <c r="M19" s="173" cm="1">
+      <c r="M19" s="170" cm="1">
         <f t="array" ref="M19">SUMPRODUCT($H$6:$H$127,(1+L19)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>2253.4467650600709</v>
       </c>
@@ -18476,7 +18473,7 @@
         <f t="shared" si="4"/>
         <v>-10000000</v>
       </c>
-      <c r="G20" s="167">
+      <c r="G20" s="164">
         <f>-IF(COUNTIF($A$6:A20,A20)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A20)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A20),0)</f>
         <v>0</v>
       </c>
@@ -18484,19 +18481,19 @@
         <f t="shared" si="5"/>
         <v>-10000000</v>
       </c>
-      <c r="J20" s="169">
+      <c r="J20" s="166">
         <f t="shared" si="0"/>
         <v>7.372283935546875E-2</v>
       </c>
-      <c r="K20" s="169">
+      <c r="K20" s="166">
         <f t="shared" si="1"/>
         <v>7.373046875E-2</v>
       </c>
-      <c r="L20" s="172">
+      <c r="L20" s="169">
         <f t="shared" si="2"/>
         <v>7.3726654052734375E-2</v>
       </c>
-      <c r="M20" s="173" cm="1">
+      <c r="M20" s="170" cm="1">
         <f t="array" ref="M20">SUMPRODUCT($H$6:$H$127,(1+L20)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>971.00612021517009</v>
       </c>
@@ -18522,7 +18519,7 @@
         <f t="shared" si="4"/>
         <v>-9400000</v>
       </c>
-      <c r="G21" s="167">
+      <c r="G21" s="164">
         <f>-IF(COUNTIF($A$6:A21,A21)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A21)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A21),0)</f>
         <v>0</v>
       </c>
@@ -18530,19 +18527,19 @@
         <f t="shared" si="5"/>
         <v>-9400000</v>
       </c>
-      <c r="J21" s="169">
+      <c r="J21" s="166">
         <f t="shared" si="0"/>
         <v>7.3726654052734375E-2</v>
       </c>
-      <c r="K21" s="169">
+      <c r="K21" s="166">
         <f t="shared" si="1"/>
         <v>7.373046875E-2</v>
       </c>
-      <c r="L21" s="172">
+      <c r="L21" s="169">
         <f t="shared" si="2"/>
         <v>7.3728561401367188E-2</v>
       </c>
-      <c r="M21" s="173" cm="1">
+      <c r="M21" s="170" cm="1">
         <f t="array" ref="M21">SUMPRODUCT($H$6:$H$127,(1+L21)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>329.80327411182225</v>
       </c>
@@ -18568,7 +18565,7 @@
         <f t="shared" si="4"/>
         <v>-2200000</v>
       </c>
-      <c r="G22" s="167">
+      <c r="G22" s="164">
         <f>-IF(COUNTIF($A$6:A22,A22)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A22)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A22),0)</f>
         <v>0</v>
       </c>
@@ -18576,19 +18573,19 @@
         <f t="shared" si="5"/>
         <v>-2200000</v>
       </c>
-      <c r="J22" s="169">
+      <c r="J22" s="166">
         <f t="shared" si="0"/>
         <v>7.3728561401367188E-2</v>
       </c>
-      <c r="K22" s="169">
+      <c r="K22" s="166">
         <f t="shared" si="1"/>
         <v>7.373046875E-2</v>
       </c>
-      <c r="L22" s="172">
+      <c r="L22" s="169">
         <f t="shared" si="2"/>
         <v>7.3729515075683594E-2</v>
       </c>
-      <c r="M22" s="173" cm="1">
+      <c r="M22" s="170" cm="1">
         <f t="array" ref="M22">SUMPRODUCT($H$6:$H$127,(1+L22)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>9.2062200084328651</v>
       </c>
@@ -18614,7 +18611,7 @@
         <f t="shared" si="4"/>
         <v>10443745</v>
       </c>
-      <c r="G23" s="167">
+      <c r="G23" s="164">
         <f>-IF(COUNTIF($A$6:A23,A23)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A23)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A23),0)</f>
         <v>0</v>
       </c>
@@ -18622,19 +18619,19 @@
         <f t="shared" si="5"/>
         <v>10443745</v>
       </c>
-      <c r="J23" s="169">
+      <c r="J23" s="166">
         <f t="shared" si="0"/>
         <v>7.3729515075683594E-2</v>
       </c>
-      <c r="K23" s="169">
+      <c r="K23" s="166">
         <f t="shared" si="1"/>
         <v>7.373046875E-2</v>
       </c>
-      <c r="L23" s="172">
+      <c r="L23" s="169">
         <f t="shared" si="2"/>
         <v>7.3729991912841797E-2</v>
       </c>
-      <c r="M23" s="173" cm="1">
+      <c r="M23" s="170" cm="1">
         <f t="array" ref="M23">SUMPRODUCT($H$6:$H$127,(1+L23)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>-151.09121477883309</v>
       </c>
@@ -18660,7 +18657,7 @@
         <f t="shared" si="4"/>
         <v>4425225</v>
       </c>
-      <c r="G24" s="167">
+      <c r="G24" s="164">
         <f>-IF(COUNTIF($A$6:A24,A24)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A24)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A24),0)</f>
         <v>0</v>
       </c>
@@ -18668,19 +18665,19 @@
         <f t="shared" si="5"/>
         <v>4425225</v>
       </c>
-      <c r="J24" s="169">
+      <c r="J24" s="166">
         <f t="shared" si="0"/>
         <v>7.3729515075683594E-2</v>
       </c>
-      <c r="K24" s="169">
+      <c r="K24" s="166">
         <f t="shared" si="1"/>
         <v>7.3729991912841797E-2</v>
       </c>
-      <c r="L24" s="172">
+      <c r="L24" s="169">
         <f t="shared" si="2"/>
         <v>7.3729753494262695E-2</v>
       </c>
-      <c r="M24" s="173" cm="1">
+      <c r="M24" s="170" cm="1">
         <f t="array" ref="M24">SUMPRODUCT($H$6:$H$127,(1+L24)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>-70.942588373553008</v>
       </c>
@@ -18706,7 +18703,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G25" s="167">
+      <c r="G25" s="164">
         <f>-IF(COUNTIF($A$6:A25,A25)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A25)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A25),0)</f>
         <v>0</v>
       </c>
@@ -18714,19 +18711,19 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="J25" s="169">
+      <c r="J25" s="166">
         <f t="shared" si="0"/>
         <v>7.3729515075683594E-2</v>
       </c>
-      <c r="K25" s="169">
+      <c r="K25" s="166">
         <f t="shared" si="1"/>
         <v>7.3729753494262695E-2</v>
       </c>
-      <c r="L25" s="172">
+      <c r="L25" s="169">
         <f t="shared" si="2"/>
         <v>7.3729634284973145E-2</v>
       </c>
-      <c r="M25" s="173" cm="1">
+      <c r="M25" s="170" cm="1">
         <f t="array" ref="M25">SUMPRODUCT($H$6:$H$127,(1+L25)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>-30.868206941056997</v>
       </c>
@@ -18752,7 +18749,7 @@
         <f t="shared" si="4"/>
         <v>-5000000</v>
       </c>
-      <c r="G26" s="167">
+      <c r="G26" s="164">
         <f>-IF(COUNTIF($A$6:A26,A26)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A26)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A26),0)</f>
         <v>0</v>
       </c>
@@ -18760,19 +18757,19 @@
         <f t="shared" si="5"/>
         <v>-5000000</v>
       </c>
-      <c r="J26" s="169">
+      <c r="J26" s="166">
         <f t="shared" si="0"/>
         <v>7.3729515075683594E-2</v>
       </c>
-      <c r="K26" s="169">
+      <c r="K26" s="166">
         <f t="shared" si="1"/>
         <v>7.3729634284973145E-2</v>
       </c>
-      <c r="L26" s="172">
+      <c r="L26" s="169">
         <f t="shared" si="2"/>
         <v>7.3729574680328369E-2</v>
       </c>
-      <c r="M26" s="173" cm="1">
+      <c r="M26" s="170" cm="1">
         <f t="array" ref="M26">SUMPRODUCT($H$6:$H$127,(1+L26)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>-10.830999140627682</v>
       </c>
@@ -18798,7 +18795,7 @@
         <f t="shared" si="4"/>
         <v>-4600000</v>
       </c>
-      <c r="G27" s="167">
+      <c r="G27" s="164">
         <f>-IF(COUNTIF($A$6:A27,A27)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A27)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A27),0)</f>
         <v>0</v>
       </c>
@@ -18806,19 +18803,19 @@
         <f t="shared" si="5"/>
         <v>-4600000</v>
       </c>
-      <c r="J27" s="169">
+      <c r="J27" s="166">
         <f t="shared" si="0"/>
         <v>7.3729515075683594E-2</v>
       </c>
-      <c r="K27" s="169">
+      <c r="K27" s="166">
         <f t="shared" si="1"/>
         <v>7.3729574680328369E-2</v>
       </c>
-      <c r="L27" s="172">
+      <c r="L27" s="169">
         <f t="shared" si="2"/>
         <v>7.3729544878005981E-2</v>
       </c>
-      <c r="M27" s="173" cm="1">
+      <c r="M27" s="170" cm="1">
         <f t="array" ref="M27">SUMPRODUCT($H$6:$H$127,(1+L27)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>-0.81239103758707643</v>
       </c>
@@ -18844,7 +18841,7 @@
         <f t="shared" si="4"/>
         <v>-10400000</v>
       </c>
-      <c r="G28" s="167">
+      <c r="G28" s="164">
         <f>-IF(COUNTIF($A$6:A28,A28)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A28)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A28),0)</f>
         <v>0</v>
       </c>
@@ -18852,19 +18849,19 @@
         <f t="shared" si="5"/>
         <v>-10400000</v>
       </c>
-      <c r="J28" s="169">
+      <c r="J28" s="166">
         <f t="shared" si="0"/>
         <v>7.3729515075683594E-2</v>
       </c>
-      <c r="K28" s="169">
+      <c r="K28" s="166">
         <f t="shared" si="1"/>
         <v>7.3729544878005981E-2</v>
       </c>
-      <c r="L28" s="172">
+      <c r="L28" s="169">
         <f t="shared" si="2"/>
         <v>7.3729529976844788E-2</v>
       </c>
-      <c r="M28" s="173" cm="1">
+      <c r="M28" s="170" cm="1">
         <f t="array" ref="M28">SUMPRODUCT($H$6:$H$127,(1+L28)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>4.1969141662120819</v>
       </c>
@@ -18890,7 +18887,7 @@
         <f t="shared" si="4"/>
         <v>3242310</v>
       </c>
-      <c r="G29" s="167">
+      <c r="G29" s="164">
         <f>-IF(COUNTIF($A$6:A29,A29)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A29)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A29),0)</f>
         <v>0</v>
       </c>
@@ -18898,19 +18895,19 @@
         <f t="shared" si="5"/>
         <v>3242310</v>
       </c>
-      <c r="J29" s="169">
+      <c r="J29" s="166">
         <f t="shared" si="0"/>
         <v>7.3729529976844788E-2</v>
       </c>
-      <c r="K29" s="169">
+      <c r="K29" s="166">
         <f t="shared" si="1"/>
         <v>7.3729544878005981E-2</v>
       </c>
-      <c r="L29" s="172">
+      <c r="L29" s="169">
         <f t="shared" si="2"/>
         <v>7.3729537427425385E-2</v>
       </c>
-      <c r="M29" s="173" cm="1">
+      <c r="M29" s="170" cm="1">
         <f t="array" ref="M29">SUMPRODUCT($H$6:$H$127,(1+L29)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>1.69226149097085</v>
       </c>
@@ -18936,7 +18933,7 @@
         <f t="shared" si="4"/>
         <v>-1745000</v>
       </c>
-      <c r="G30" s="167">
+      <c r="G30" s="164">
         <f>-IF(COUNTIF($A$6:A30,A30)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A30)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A30),0)</f>
         <v>0</v>
       </c>
@@ -18944,19 +18941,19 @@
         <f t="shared" si="5"/>
         <v>-1745000</v>
       </c>
-      <c r="J30" s="169">
+      <c r="J30" s="166">
         <f t="shared" si="0"/>
         <v>7.3729537427425385E-2</v>
       </c>
-      <c r="K30" s="169">
+      <c r="K30" s="166">
         <f t="shared" si="1"/>
         <v>7.3729544878005981E-2</v>
       </c>
-      <c r="L30" s="172">
+      <c r="L30" s="169">
         <f t="shared" si="2"/>
         <v>7.3729541152715683E-2</v>
       </c>
-      <c r="M30" s="173" cm="1">
+      <c r="M30" s="170" cm="1">
         <f t="array" ref="M30">SUMPRODUCT($H$6:$H$127,(1+L30)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>0.43993529584258795</v>
       </c>
@@ -18982,7 +18979,7 @@
         <f t="shared" si="4"/>
         <v>-4600000</v>
       </c>
-      <c r="G31" s="167">
+      <c r="G31" s="164">
         <f>-IF(COUNTIF($A$6:A31,A31)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A31)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A31),0)</f>
         <v>0</v>
       </c>
@@ -18990,19 +18987,19 @@
         <f t="shared" si="5"/>
         <v>-4600000</v>
       </c>
-      <c r="J31" s="169">
+      <c r="J31" s="166">
         <f t="shared" si="0"/>
         <v>7.3729541152715683E-2</v>
       </c>
-      <c r="K31" s="169">
+      <c r="K31" s="166">
         <f t="shared" si="1"/>
         <v>7.3729544878005981E-2</v>
       </c>
-      <c r="L31" s="172">
+      <c r="L31" s="169">
         <f t="shared" si="2"/>
         <v>7.3729543015360832E-2</v>
       </c>
-      <c r="M31" s="173" cm="1">
+      <c r="M31" s="170" cm="1">
         <f t="array" ref="M31">SUMPRODUCT($H$6:$H$127,(1+L31)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>-0.18622785620391369</v>
       </c>
@@ -19028,7 +19025,7 @@
         <f t="shared" si="4"/>
         <v>-6000000</v>
       </c>
-      <c r="G32" s="167">
+      <c r="G32" s="164">
         <f>-IF(COUNTIF($A$6:A32,A32)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A32)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A32),0)</f>
         <v>0</v>
       </c>
@@ -19036,19 +19033,19 @@
         <f t="shared" si="5"/>
         <v>-6000000</v>
       </c>
-      <c r="J32" s="169">
+      <c r="J32" s="166">
         <f t="shared" si="0"/>
         <v>7.3729541152715683E-2</v>
       </c>
-      <c r="K32" s="169">
+      <c r="K32" s="166">
         <f t="shared" si="1"/>
         <v>7.3729543015360832E-2</v>
       </c>
-      <c r="L32" s="172">
+      <c r="L32" s="169">
         <f t="shared" si="2"/>
         <v>7.3729542084038258E-2</v>
       </c>
-      <c r="M32" s="173" cm="1">
+      <c r="M32" s="170" cm="1">
         <f t="array" ref="M32">SUMPRODUCT($H$6:$H$127,(1+L32)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>0.12685369048267603</v>
       </c>
@@ -19074,7 +19071,7 @@
         <f t="shared" si="4"/>
         <v>-1855000</v>
       </c>
-      <c r="G33" s="167">
+      <c r="G33" s="164">
         <f>-IF(COUNTIF($A$6:A33,A33)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A33)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A33),0)</f>
         <v>0</v>
       </c>
@@ -19082,19 +19079,19 @@
         <f t="shared" si="5"/>
         <v>-1855000</v>
       </c>
-      <c r="J33" s="169">
+      <c r="J33" s="166">
         <f t="shared" si="0"/>
         <v>7.3729542084038258E-2</v>
       </c>
-      <c r="K33" s="169">
+      <c r="K33" s="166">
         <f t="shared" si="1"/>
         <v>7.3729543015360832E-2</v>
       </c>
-      <c r="L33" s="172">
+      <c r="L33" s="169">
         <f t="shared" si="2"/>
         <v>7.3729542549699545E-2</v>
       </c>
-      <c r="M33" s="173" cm="1">
+      <c r="M33" s="170" cm="1">
         <f t="array" ref="M33">SUMPRODUCT($H$6:$H$127,(1+L33)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>-2.968704467639327E-2</v>
       </c>
@@ -19120,7 +19117,7 @@
         <f t="shared" si="4"/>
         <v>4087330</v>
       </c>
-      <c r="G34" s="167">
+      <c r="G34" s="164">
         <f>-IF(COUNTIF($A$6:A34,A34)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A34)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A34),0)</f>
         <v>0</v>
       </c>
@@ -19128,19 +19125,19 @@
         <f t="shared" si="5"/>
         <v>4087330</v>
       </c>
-      <c r="J34" s="169">
+      <c r="J34" s="166">
         <f t="shared" si="0"/>
         <v>7.3729542084038258E-2</v>
       </c>
-      <c r="K34" s="169">
+      <c r="K34" s="166">
         <f t="shared" si="1"/>
         <v>7.3729542549699545E-2</v>
       </c>
-      <c r="L34" s="172">
+      <c r="L34" s="169">
         <f t="shared" si="2"/>
         <v>7.3729542316868901E-2</v>
       </c>
-      <c r="M34" s="173" cm="1">
+      <c r="M34" s="170" cm="1">
         <f t="array" ref="M34">SUMPRODUCT($H$6:$H$127,(1+L34)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>4.8583300318568945E-2</v>
       </c>
@@ -19166,7 +19163,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G35" s="167">
+      <c r="G35" s="164">
         <f>-IF(COUNTIF($A$6:A35,A35)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A35)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A35),0)</f>
         <v>-1128907</v>
       </c>
@@ -19174,19 +19171,19 @@
         <f t="shared" si="5"/>
         <v>-1128907</v>
       </c>
-      <c r="J35" s="169">
+      <c r="J35" s="166">
         <f t="shared" si="0"/>
         <v>7.3729542316868901E-2</v>
       </c>
-      <c r="K35" s="169">
+      <c r="K35" s="166">
         <f t="shared" si="1"/>
         <v>7.3729542549699545E-2</v>
       </c>
-      <c r="L35" s="172">
+      <c r="L35" s="169">
         <f t="shared" si="2"/>
         <v>7.3729542433284223E-2</v>
       </c>
-      <c r="M35" s="173" cm="1">
+      <c r="M35" s="170" cm="1">
         <f t="array" ref="M35">SUMPRODUCT($H$6:$H$127,(1+L35)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>9.4481273554265499E-3</v>
       </c>
@@ -19212,7 +19209,7 @@
         <f t="shared" si="4"/>
         <v>1923105</v>
       </c>
-      <c r="G36" s="167">
+      <c r="G36" s="164">
         <f>-IF(COUNTIF($A$6:A36,A36)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A36)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A36),0)</f>
         <v>0</v>
       </c>
@@ -19220,19 +19217,19 @@
         <f t="shared" si="5"/>
         <v>1923105</v>
       </c>
-      <c r="J36" s="169">
+      <c r="J36" s="166">
         <f t="shared" si="0"/>
         <v>7.3729542433284223E-2</v>
       </c>
-      <c r="K36" s="169">
+      <c r="K36" s="166">
         <f t="shared" si="1"/>
         <v>7.3729542549699545E-2</v>
       </c>
-      <c r="L36" s="172">
+      <c r="L36" s="169">
         <f t="shared" si="2"/>
         <v>7.3729542491491884E-2</v>
       </c>
-      <c r="M36" s="173" cm="1">
+      <c r="M36" s="170" cm="1">
         <f t="array" ref="M36">SUMPRODUCT($H$6:$H$127,(1+L36)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>-1.0119525715708733E-2</v>
       </c>
@@ -19258,7 +19255,7 @@
         <f t="shared" si="4"/>
         <v>679120</v>
       </c>
-      <c r="G37" s="167">
+      <c r="G37" s="164">
         <f>-IF(COUNTIF($A$6:A37,A37)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A37)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A37),0)</f>
         <v>0</v>
       </c>
@@ -19266,19 +19263,19 @@
         <f t="shared" si="5"/>
         <v>679120</v>
       </c>
-      <c r="J37" s="169">
+      <c r="J37" s="166">
         <f t="shared" si="0"/>
         <v>7.3729542433284223E-2</v>
       </c>
-      <c r="K37" s="169">
+      <c r="K37" s="166">
         <f t="shared" si="1"/>
         <v>7.3729542491491884E-2</v>
       </c>
-      <c r="L37" s="172">
+      <c r="L37" s="169">
         <f t="shared" si="2"/>
         <v>7.3729542462388054E-2</v>
       </c>
-      <c r="M37" s="173" cm="1">
+      <c r="M37" s="170" cm="1">
         <f t="array" ref="M37">SUMPRODUCT($H$6:$H$127,(1+L37)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>-3.3571384847164154E-4</v>
       </c>
@@ -19304,7 +19301,7 @@
         <f t="shared" ref="E38:E69" si="7">C38-D38</f>
         <v>-4000000</v>
       </c>
-      <c r="G38" s="167">
+      <c r="G38" s="164">
         <f>-IF(COUNTIF($A$6:A38,A38)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A38)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A38),0)</f>
         <v>0</v>
       </c>
@@ -19312,19 +19309,19 @@
         <f t="shared" si="5"/>
         <v>-4000000</v>
       </c>
-      <c r="J38" s="169">
+      <c r="J38" s="166">
         <f t="shared" si="0"/>
         <v>7.3729542433284223E-2</v>
       </c>
-      <c r="K38" s="169">
+      <c r="K38" s="166">
         <f t="shared" si="1"/>
         <v>7.3729542462388054E-2</v>
       </c>
-      <c r="L38" s="172">
+      <c r="L38" s="169">
         <f t="shared" si="2"/>
         <v>7.3729542447836138E-2</v>
       </c>
-      <c r="M38" s="173" cm="1">
+      <c r="M38" s="170" cm="1">
         <f t="array" ref="M38">SUMPRODUCT($H$6:$H$127,(1+L38)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>4.5562591403722763E-3</v>
       </c>
@@ -19350,7 +19347,7 @@
         <f t="shared" si="7"/>
         <v>998970.04</v>
       </c>
-      <c r="G39" s="167">
+      <c r="G39" s="164">
         <f>-IF(COUNTIF($A$6:A39,A39)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A39)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A39),0)</f>
         <v>0</v>
       </c>
@@ -19358,19 +19355,19 @@
         <f t="shared" si="5"/>
         <v>998970.04</v>
       </c>
-      <c r="J39" s="169">
+      <c r="J39" s="166">
         <f t="shared" si="0"/>
         <v>7.3729542447836138E-2</v>
       </c>
-      <c r="K39" s="169">
+      <c r="K39" s="166">
         <f t="shared" si="1"/>
         <v>7.3729542462388054E-2</v>
       </c>
-      <c r="L39" s="172">
+      <c r="L39" s="169">
         <f t="shared" si="2"/>
         <v>7.3729542455112096E-2</v>
       </c>
-      <c r="M39" s="173" cm="1">
+      <c r="M39" s="170" cm="1">
         <f t="array" ref="M39">SUMPRODUCT($H$6:$H$127,(1+L39)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>2.1103173494338989E-3</v>
       </c>
@@ -19396,7 +19393,7 @@
         <f t="shared" si="7"/>
         <v>2368545</v>
       </c>
-      <c r="G40" s="167">
+      <c r="G40" s="164">
         <f>-IF(COUNTIF($A$6:A40,A40)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A40)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A40),0)</f>
         <v>-1148907</v>
       </c>
@@ -19404,19 +19401,19 @@
         <f t="shared" si="5"/>
         <v>1219638</v>
       </c>
-      <c r="J40" s="169">
+      <c r="J40" s="166">
         <f t="shared" si="0"/>
         <v>7.3729542455112096E-2</v>
       </c>
-      <c r="K40" s="169">
+      <c r="K40" s="166">
         <f t="shared" si="1"/>
         <v>7.3729542462388054E-2</v>
       </c>
-      <c r="L40" s="172">
+      <c r="L40" s="169">
         <f t="shared" si="2"/>
         <v>7.3729542458750075E-2</v>
       </c>
-      <c r="M40" s="173" cm="1">
+      <c r="M40" s="170" cm="1">
         <f t="array" ref="M40">SUMPRODUCT($H$6:$H$127,(1+L40)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>8.8723422959446907E-4</v>
       </c>
@@ -19442,7 +19439,7 @@
         <f t="shared" si="7"/>
         <v>-3191939.24</v>
       </c>
-      <c r="G41" s="167">
+      <c r="G41" s="164">
         <f>-IF(COUNTIF($A$6:A41,A41)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A41)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A41),0)</f>
         <v>0</v>
       </c>
@@ -19450,19 +19447,19 @@
         <f t="shared" si="5"/>
         <v>-3191939.24</v>
       </c>
-      <c r="J41" s="169">
+      <c r="J41" s="166">
         <f t="shared" si="0"/>
         <v>7.3729542458750075E-2</v>
       </c>
-      <c r="K41" s="169">
+      <c r="K41" s="166">
         <f t="shared" si="1"/>
         <v>7.3729542462388054E-2</v>
       </c>
-      <c r="L41" s="172">
+      <c r="L41" s="169">
         <f t="shared" si="2"/>
         <v>7.3729542460569064E-2</v>
       </c>
-      <c r="M41" s="173" cm="1">
+      <c r="M41" s="170" cm="1">
         <f t="array" ref="M41">SUMPRODUCT($H$6:$H$127,(1+L41)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>2.7578230947256088E-4</v>
       </c>
@@ -19488,7 +19485,7 @@
         <f t="shared" si="7"/>
         <v>-1076405.04</v>
       </c>
-      <c r="G42" s="167">
+      <c r="G42" s="164">
         <f>-IF(COUNTIF($A$6:A42,A42)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A42)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A42),0)</f>
         <v>0</v>
       </c>
@@ -19496,19 +19493,19 @@
         <f t="shared" si="5"/>
         <v>-1076405.04</v>
       </c>
-      <c r="J42" s="169">
+      <c r="J42" s="166">
         <f t="shared" si="0"/>
         <v>7.3729542460569064E-2</v>
       </c>
-      <c r="K42" s="169">
+      <c r="K42" s="166">
         <f t="shared" si="1"/>
         <v>7.3729542462388054E-2</v>
       </c>
-      <c r="L42" s="172">
+      <c r="L42" s="169">
         <f t="shared" si="2"/>
         <v>7.3729542461478559E-2</v>
       </c>
-      <c r="M42" s="173" cm="1">
+      <c r="M42" s="170" cm="1">
         <f t="array" ref="M42">SUMPRODUCT($H$6:$H$127,(1+L42)^(-($A$6:$A$127-$A$6)/365))</f>
         <v>-2.9958318918943405E-5</v>
       </c>
@@ -19534,7 +19531,7 @@
         <f t="shared" si="7"/>
         <v>3048706.28</v>
       </c>
-      <c r="G43" s="167">
+      <c r="G43" s="164">
         <f>-IF(COUNTIF($A$6:A43,A43)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A43)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A43),0)</f>
         <v>0</v>
       </c>
@@ -19564,7 +19561,7 @@
         <f t="shared" si="7"/>
         <v>-2000000</v>
       </c>
-      <c r="G44" s="167">
+      <c r="G44" s="164">
         <f>-IF(COUNTIF($A$6:A44,A44)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A44)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A44),0)</f>
         <v>0</v>
       </c>
@@ -19594,7 +19591,7 @@
         <f t="shared" si="7"/>
         <v>450000</v>
       </c>
-      <c r="G45" s="167">
+      <c r="G45" s="164">
         <f>-IF(COUNTIF($A$6:A45,A45)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A45)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A45),0)</f>
         <v>0</v>
       </c>
@@ -19624,7 +19621,7 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="G46" s="167">
+      <c r="G46" s="164">
         <f>-IF(COUNTIF($A$6:A46,A46)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A46)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A46),0)</f>
         <v>0</v>
       </c>
@@ -19654,7 +19651,7 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="G47" s="167">
+      <c r="G47" s="164">
         <f>-IF(COUNTIF($A$6:A47,A47)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A47)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A47),0)</f>
         <v>0</v>
       </c>
@@ -19684,7 +19681,7 @@
         <f t="shared" si="7"/>
         <v>450000</v>
       </c>
-      <c r="G48" s="167">
+      <c r="G48" s="164">
         <f>-IF(COUNTIF($A$6:A48,A48)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A48)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A48),0)</f>
         <v>0</v>
       </c>
@@ -19714,7 +19711,7 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="G49" s="167">
+      <c r="G49" s="164">
         <f>-IF(COUNTIF($A$6:A49,A49)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A49)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A49),0)</f>
         <v>0</v>
       </c>
@@ -19744,7 +19741,7 @@
         <f t="shared" si="7"/>
         <v>2819720</v>
       </c>
-      <c r="G50" s="167">
+      <c r="G50" s="164">
         <f>-IF(COUNTIF($A$6:A50,A50)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A50)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A50),0)</f>
         <v>0</v>
       </c>
@@ -19774,7 +19771,7 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="G51" s="167">
+      <c r="G51" s="164">
         <f>-IF(COUNTIF($A$6:A51,A51)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A51)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A51),0)</f>
         <v>0</v>
       </c>
@@ -19804,7 +19801,7 @@
         <f t="shared" si="7"/>
         <v>853874.94</v>
       </c>
-      <c r="G52" s="167">
+      <c r="G52" s="164">
         <f>-IF(COUNTIF($A$6:A52,A52)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A52)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A52),0)</f>
         <v>0</v>
       </c>
@@ -19834,7 +19831,7 @@
         <f t="shared" si="7"/>
         <v>-1917460</v>
       </c>
-      <c r="G53" s="167">
+      <c r="G53" s="164">
         <f>-IF(COUNTIF($A$6:A53,A53)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A53)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A53),0)</f>
         <v>-1196593</v>
       </c>
@@ -19864,7 +19861,7 @@
         <f t="shared" si="7"/>
         <v>4000000</v>
       </c>
-      <c r="G54" s="167">
+      <c r="G54" s="164">
         <f>-IF(COUNTIF($A$6:A54,A54)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A54)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A54),0)</f>
         <v>0</v>
       </c>
@@ -19894,7 +19891,7 @@
         <f t="shared" si="7"/>
         <v>1945790.17</v>
       </c>
-      <c r="G55" s="167">
+      <c r="G55" s="164">
         <f>-IF(COUNTIF($A$6:A55,A55)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A55)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A55),0)</f>
         <v>0</v>
       </c>
@@ -19924,7 +19921,7 @@
         <f t="shared" si="7"/>
         <v>-1000000</v>
       </c>
-      <c r="G56" s="167">
+      <c r="G56" s="164">
         <f>-IF(COUNTIF($A$6:A56,A56)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A56)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A56),0)</f>
         <v>-1113907</v>
       </c>
@@ -19954,7 +19951,7 @@
         <f t="shared" si="7"/>
         <v>38288179.109999999</v>
       </c>
-      <c r="G57" s="167">
+      <c r="G57" s="164">
         <f>-IF(COUNTIF($A$6:A57,A57)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A57)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A57),0)</f>
         <v>0</v>
       </c>
@@ -19984,7 +19981,7 @@
         <f t="shared" si="7"/>
         <v>5747034.3099999996</v>
       </c>
-      <c r="G58" s="167">
+      <c r="G58" s="164">
         <f>-IF(COUNTIF($A$6:A58,A58)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A58)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A58),0)</f>
         <v>-31500</v>
       </c>
@@ -20014,7 +20011,7 @@
         <f t="shared" si="7"/>
         <v>2480910.0099999998</v>
       </c>
-      <c r="G59" s="167">
+      <c r="G59" s="164">
         <f>-IF(COUNTIF($A$6:A59,A59)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A59)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A59),0)</f>
         <v>0</v>
       </c>
@@ -20044,7 +20041,7 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="G60" s="167">
+      <c r="G60" s="164">
         <f>-IF(COUNTIF($A$6:A60,A60)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A60)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A60),0)</f>
         <v>-1123907</v>
       </c>
@@ -20074,7 +20071,7 @@
         <f t="shared" si="7"/>
         <v>3169354.38</v>
       </c>
-      <c r="G61" s="167">
+      <c r="G61" s="164">
         <f>-IF(COUNTIF($A$6:A61,A61)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A61)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A61),0)</f>
         <v>0</v>
       </c>
@@ -20104,7 +20101,7 @@
         <f t="shared" si="7"/>
         <v>1988729.65</v>
       </c>
-      <c r="G62" s="167">
+      <c r="G62" s="164">
         <f>-IF(COUNTIF($A$6:A62,A62)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A62)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A62),0)</f>
         <v>0</v>
       </c>
@@ -20134,7 +20131,7 @@
         <f t="shared" si="7"/>
         <v>17154800</v>
       </c>
-      <c r="G63" s="167">
+      <c r="G63" s="164">
         <f>-IF(COUNTIF($A$6:A63,A63)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A63)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A63),0)</f>
         <v>0</v>
       </c>
@@ -20164,7 +20161,7 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="G64" s="167">
+      <c r="G64" s="164">
         <f>-IF(COUNTIF($A$6:A64,A64)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A64)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A64),0)</f>
         <v>-1219376.3500000001</v>
       </c>
@@ -20194,7 +20191,7 @@
         <f t="shared" si="7"/>
         <v>7609365.8300000001</v>
       </c>
-      <c r="G65" s="167">
+      <c r="G65" s="164">
         <f>-IF(COUNTIF($A$6:A65,A65)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A65)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A65),0)</f>
         <v>0</v>
       </c>
@@ -20224,7 +20221,7 @@
         <f t="shared" si="7"/>
         <v>948648</v>
       </c>
-      <c r="G66" s="167">
+      <c r="G66" s="164">
         <f>-IF(COUNTIF($A$6:A66,A66)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A66)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A66),0)</f>
         <v>-2112239.5833333302</v>
       </c>
@@ -20254,7 +20251,7 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="G67" s="167">
+      <c r="G67" s="164">
         <f>-IF(COUNTIF($A$6:A67,A67)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A67)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A67),0)</f>
         <v>-1747249.58333333</v>
       </c>
@@ -20284,7 +20281,7 @@
         <f t="shared" si="7"/>
         <v>3798648.74</v>
       </c>
-      <c r="G68" s="167">
+      <c r="G68" s="164">
         <f>-IF(COUNTIF($A$6:A68,A68)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A68)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A68),0)</f>
         <v>-1709656.25</v>
       </c>
@@ -20314,7 +20311,7 @@
         <f t="shared" si="7"/>
         <v>7240475.3200000003</v>
       </c>
-      <c r="G69" s="167">
+      <c r="G69" s="164">
         <f>-IF(COUNTIF($A$6:A69,A69)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A69)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A69),0)</f>
         <v>0</v>
       </c>
@@ -20344,7 +20341,7 @@
         <f t="shared" ref="E70:E101" si="9">C70-D70</f>
         <v>954998.58</v>
       </c>
-      <c r="G70" s="167">
+      <c r="G70" s="164">
         <f>-IF(COUNTIF($A$6:A70,A70)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A70)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A70),0)</f>
         <v>0</v>
       </c>
@@ -20374,7 +20371,7 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="G71" s="167">
+      <c r="G71" s="164">
         <f>-IF(COUNTIF($A$6:A71,A71)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A71)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A71),0)</f>
         <v>0</v>
       </c>
@@ -20404,7 +20401,7 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="G72" s="167">
+      <c r="G72" s="164">
         <f>-IF(COUNTIF($A$6:A72,A72)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A72)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A72),0)</f>
         <v>-1818214.7</v>
       </c>
@@ -20434,7 +20431,7 @@
         <f t="shared" si="9"/>
         <v>476082</v>
       </c>
-      <c r="G73" s="167">
+      <c r="G73" s="164">
         <f>-IF(COUNTIF($A$6:A73,A73)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A73)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A73),0)</f>
         <v>0</v>
       </c>
@@ -20464,7 +20461,7 @@
         <f t="shared" si="9"/>
         <v>1152462.5</v>
       </c>
-      <c r="G74" s="167">
+      <c r="G74" s="164">
         <f>-IF(COUNTIF($A$6:A74,A74)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A74)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A74),0)</f>
         <v>-1734656.25</v>
       </c>
@@ -20494,7 +20491,7 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="G75" s="167">
+      <c r="G75" s="164">
         <f>-IF(COUNTIF($A$6:A75,A75)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A75)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A75),0)</f>
         <v>0</v>
       </c>
@@ -20524,7 +20521,7 @@
         <f t="shared" si="9"/>
         <v>737907.5</v>
       </c>
-      <c r="G76" s="167">
+      <c r="G76" s="164">
         <f>-IF(COUNTIF($A$6:A76,A76)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A76)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A76),0)</f>
         <v>-1717706.25</v>
       </c>
@@ -20554,7 +20551,7 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="G77" s="167">
+      <c r="G77" s="164">
         <f>-IF(COUNTIF($A$6:A77,A77)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A77)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A77),0)</f>
         <v>0</v>
       </c>
@@ -20584,7 +20581,7 @@
         <f t="shared" si="9"/>
         <v>3481490.1</v>
       </c>
-      <c r="G78" s="167">
+      <c r="G78" s="164">
         <f>-IF(COUNTIF($A$6:A78,A78)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A78)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A78),0)</f>
         <v>0</v>
       </c>
@@ -20614,7 +20611,7 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="G79" s="167">
+      <c r="G79" s="164">
         <f>-IF(COUNTIF($A$6:A79,A79)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A79)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A79),0)</f>
         <v>0</v>
       </c>
@@ -20644,7 +20641,7 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="G80" s="167">
+      <c r="G80" s="164">
         <f>-IF(COUNTIF($A$6:A80,A80)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A80)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A80),0)</f>
         <v>-1719656.25</v>
       </c>
@@ -20674,7 +20671,7 @@
         <f t="shared" si="9"/>
         <v>-5500000</v>
       </c>
-      <c r="G81" s="167">
+      <c r="G81" s="164">
         <f>-IF(COUNTIF($A$6:A81,A81)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A81)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A81),0)</f>
         <v>0</v>
       </c>
@@ -20704,7 +20701,7 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="G82" s="167">
+      <c r="G82" s="164">
         <f>-IF(COUNTIF($A$6:A82,A82)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A82)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A82),0)</f>
         <v>-1955318.75</v>
       </c>
@@ -20734,7 +20731,7 @@
         <f t="shared" si="9"/>
         <v>-7000000</v>
       </c>
-      <c r="G83" s="167">
+      <c r="G83" s="164">
         <f>-IF(COUNTIF($A$6:A83,A83)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A83)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A83),0)</f>
         <v>0</v>
       </c>
@@ -20764,7 +20761,7 @@
         <f t="shared" si="9"/>
         <v>694476.87</v>
       </c>
-      <c r="G84" s="167">
+      <c r="G84" s="164">
         <f>-IF(COUNTIF($A$6:A84,A84)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A84)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A84),0)</f>
         <v>-847503.40312499995</v>
       </c>
@@ -20794,7 +20791,7 @@
         <f t="shared" si="9"/>
         <v>6288799.3899999997</v>
       </c>
-      <c r="G85" s="167">
+      <c r="G85" s="164">
         <f>-IF(COUNTIF($A$6:A85,A85)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A85)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A85),0)</f>
         <v>0</v>
       </c>
@@ -20824,7 +20821,7 @@
         <f t="shared" si="9"/>
         <v>451182.19</v>
       </c>
-      <c r="G86" s="167">
+      <c r="G86" s="164">
         <f>-IF(COUNTIF($A$6:A86,A86)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A86)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A86),0)</f>
         <v>0</v>
       </c>
@@ -20854,7 +20851,7 @@
         <f t="shared" si="9"/>
         <v>1064625.1000000001</v>
       </c>
-      <c r="G87" s="167">
+      <c r="G87" s="164">
         <f>-IF(COUNTIF($A$6:A87,A87)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A87)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A87),0)</f>
         <v>0</v>
       </c>
@@ -20884,7 +20881,7 @@
         <f t="shared" si="9"/>
         <v>-6000000</v>
       </c>
-      <c r="G88" s="167">
+      <c r="G88" s="164">
         <f>-IF(COUNTIF($A$6:A88,A88)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A88)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A88),0)</f>
         <v>-374241.19968750002</v>
       </c>
@@ -20914,7 +20911,7 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="G89" s="167">
+      <c r="G89" s="164">
         <f>-IF(COUNTIF($A$6:A89,A89)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A89)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A89),0)</f>
         <v>-6152916.6603124999</v>
       </c>
@@ -20944,7 +20941,7 @@
         <f t="shared" si="9"/>
         <v>-2500000</v>
       </c>
-      <c r="G90" s="167">
+      <c r="G90" s="164">
         <f>-IF(COUNTIF($A$6:A90,A90)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A90)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A90),0)</f>
         <v>0</v>
       </c>
@@ -20974,7 +20971,7 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="G91" s="167">
+      <c r="G91" s="164">
         <f>-IF(COUNTIF($A$6:A91,A91)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A91)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A91),0)</f>
         <v>0</v>
       </c>
@@ -21004,7 +21001,7 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="G92" s="167">
+      <c r="G92" s="164">
         <f>-IF(COUNTIF($A$6:A92,A92)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A92)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A92),0)</f>
         <v>-3283946.75</v>
       </c>
@@ -21034,7 +21031,7 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="G93" s="167">
+      <c r="G93" s="164">
         <f>-IF(COUNTIF($A$6:A93,A93)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A93)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A93),0)</f>
         <v>0</v>
       </c>
@@ -21064,7 +21061,7 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="G94" s="167">
+      <c r="G94" s="164">
         <f>-IF(COUNTIF($A$6:A94,A94)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A94)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A94),0)</f>
         <v>-3662054</v>
       </c>
@@ -21094,7 +21091,7 @@
         <f t="shared" si="9"/>
         <v>-3600000</v>
       </c>
-      <c r="G95" s="167">
+      <c r="G95" s="164">
         <f>-IF(COUNTIF($A$6:A95,A95)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A95)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A95),0)</f>
         <v>0</v>
       </c>
@@ -21124,7 +21121,7 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="G96" s="167">
+      <c r="G96" s="164">
         <f>-IF(COUNTIF($A$6:A96,A96)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A96)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A96),0)</f>
         <v>-404800.68224062503</v>
       </c>
@@ -21154,7 +21151,7 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="G97" s="167">
+      <c r="G97" s="164">
         <f>-IF(COUNTIF($A$6:A97,A97)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A97)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A97),0)</f>
         <v>0</v>
       </c>
@@ -21184,7 +21181,7 @@
         <f t="shared" si="9"/>
         <v>-9751000</v>
       </c>
-      <c r="G98" s="167">
+      <c r="G98" s="164">
         <f>-IF(COUNTIF($A$6:A98,A98)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A98)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A98),0)</f>
         <v>0</v>
       </c>
@@ -21214,7 +21211,7 @@
         <f t="shared" si="9"/>
         <v>-500000</v>
       </c>
-      <c r="G99" s="167">
+      <c r="G99" s="164">
         <f>-IF(COUNTIF($A$6:A99,A99)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A99)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A99),0)</f>
         <v>0</v>
       </c>
@@ -21244,7 +21241,7 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="G100" s="167">
+      <c r="G100" s="164">
         <f>-IF(COUNTIF($A$6:A100,A100)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A100)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A100),0)</f>
         <v>0</v>
       </c>
@@ -21274,7 +21271,7 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="G101" s="167">
+      <c r="G101" s="164">
         <f>-IF(COUNTIF($A$6:A101,A101)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A101)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A101),0)</f>
         <v>-2704040.38416667</v>
       </c>
@@ -21304,7 +21301,7 @@
         <f t="shared" ref="E102:E126" si="12">C102-D102</f>
         <v>-4700000</v>
       </c>
-      <c r="G102" s="167">
+      <c r="G102" s="164">
         <f>-IF(COUNTIF($A$6:A102,A102)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A102)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A102),0)</f>
         <v>0</v>
       </c>
@@ -21334,7 +21331,7 @@
         <f t="shared" si="12"/>
         <v>-13500000</v>
       </c>
-      <c r="G103" s="167">
+      <c r="G103" s="164">
         <f>-IF(COUNTIF($A$6:A103,A103)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A103)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A103),0)</f>
         <v>0</v>
       </c>
@@ -21364,7 +21361,7 @@
         <f t="shared" si="12"/>
         <v>-1500000</v>
       </c>
-      <c r="G104" s="167">
+      <c r="G104" s="164">
         <f>-IF(COUNTIF($A$6:A104,A104)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A104)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A104),0)</f>
         <v>-1779108.5649999999</v>
       </c>
@@ -21394,7 +21391,7 @@
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="G105" s="167">
+      <c r="G105" s="164">
         <f>-IF(COUNTIF($A$6:A105,A105)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A105)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A105),0)</f>
         <v>0</v>
       </c>
@@ -21424,7 +21421,7 @@
         <f t="shared" si="12"/>
         <v>-3640000</v>
       </c>
-      <c r="G106" s="167">
+      <c r="G106" s="164">
         <f>-IF(COUNTIF($A$6:A106,A106)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A106)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A106),0)</f>
         <v>0</v>
       </c>
@@ -21454,7 +21451,7 @@
         <f t="shared" si="12"/>
         <v>-7400000</v>
       </c>
-      <c r="G107" s="167">
+      <c r="G107" s="164">
         <f>-IF(COUNTIF($A$6:A107,A107)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A107)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A107),0)</f>
         <v>0</v>
       </c>
@@ -21484,7 +21481,7 @@
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="G108" s="167">
+      <c r="G108" s="164">
         <f>-IF(COUNTIF($A$6:A108,A108)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A108)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A108),0)</f>
         <v>-2044496.29333333</v>
       </c>
@@ -21514,7 +21511,7 @@
         <f t="shared" si="12"/>
         <v>-7000000</v>
       </c>
-      <c r="G109" s="167">
+      <c r="G109" s="164">
         <f>-IF(COUNTIF($A$6:A109,A109)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A109)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A109),0)</f>
         <v>0</v>
       </c>
@@ -21544,7 +21541,7 @@
         <f t="shared" si="12"/>
         <v>-13000000</v>
       </c>
-      <c r="G110" s="167">
+      <c r="G110" s="164">
         <f>-IF(COUNTIF($A$6:A110,A110)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A110)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A110),0)</f>
         <v>0</v>
       </c>
@@ -21574,7 +21571,7 @@
         <f t="shared" si="12"/>
         <v>24000000</v>
       </c>
-      <c r="G111" s="167">
+      <c r="G111" s="164">
         <f>-IF(COUNTIF($A$6:A111,A111)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A111)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A111),0)</f>
         <v>0</v>
       </c>
@@ -21604,7 +21601,7 @@
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="G112" s="167">
+      <c r="G112" s="164">
         <f>-IF(COUNTIF($A$6:A112,A112)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A112)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A112),0)</f>
         <v>0</v>
       </c>
@@ -21634,7 +21631,7 @@
         <f t="shared" si="12"/>
         <v>-2260000</v>
       </c>
-      <c r="G113" s="167">
+      <c r="G113" s="164">
         <f>-IF(COUNTIF($A$6:A113,A113)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A113)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A113),0)</f>
         <v>0</v>
       </c>
@@ -21664,7 +21661,7 @@
         <f t="shared" si="12"/>
         <v>-10750000</v>
       </c>
-      <c r="G114" s="167">
+      <c r="G114" s="164">
         <f>-IF(COUNTIF($A$6:A114,A114)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A114)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A114),0)</f>
         <v>0</v>
       </c>
@@ -21694,7 +21691,7 @@
         <f t="shared" si="12"/>
         <v>-13600000</v>
       </c>
-      <c r="G115" s="167">
+      <c r="G115" s="164">
         <f>-IF(COUNTIF($A$6:A115,A115)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A115)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A115),0)</f>
         <v>0</v>
       </c>
@@ -21724,7 +21721,7 @@
         <f t="shared" si="12"/>
         <v>-1209348.2</v>
       </c>
-      <c r="G116" s="167">
+      <c r="G116" s="164">
         <f>-IF(COUNTIF($A$6:A116,A116)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A116)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A116),0)</f>
         <v>0</v>
       </c>
@@ -21754,7 +21751,7 @@
         <f t="shared" si="12"/>
         <v>-4614366</v>
       </c>
-      <c r="G117" s="167">
+      <c r="G117" s="164">
         <f>-IF(COUNTIF($A$6:A117,A117)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A117)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A117),0)</f>
         <v>0</v>
       </c>
@@ -21784,7 +21781,7 @@
         <f t="shared" si="12"/>
         <v>-8000000</v>
       </c>
-      <c r="G118" s="167">
+      <c r="G118" s="164">
         <f>-IF(COUNTIF($A$6:A118,A118)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A118)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A118),0)</f>
         <v>0</v>
       </c>
@@ -21814,7 +21811,7 @@
         <f t="shared" si="12"/>
         <v>-1959878.2</v>
       </c>
-      <c r="G119" s="167">
+      <c r="G119" s="164">
         <f>-IF(COUNTIF($A$6:A119,A119)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A119)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A119),0)</f>
         <v>0</v>
       </c>
@@ -21844,7 +21841,7 @@
         <f t="shared" si="12"/>
         <v>-1219884.74</v>
       </c>
-      <c r="G120" s="167">
+      <c r="G120" s="164">
         <f>-IF(COUNTIF($A$6:A120,A120)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A120)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A120),0)</f>
         <v>0</v>
       </c>
@@ -21874,7 +21871,7 @@
         <f t="shared" si="12"/>
         <v>-1672749.65</v>
       </c>
-      <c r="G121" s="167">
+      <c r="G121" s="164">
         <f>-IF(COUNTIF($A$6:A121,A121)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A121)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A121),0)</f>
         <v>0</v>
       </c>
@@ -21904,7 +21901,7 @@
         <f t="shared" si="12"/>
         <v>-3000000</v>
       </c>
-      <c r="G122" s="167">
+      <c r="G122" s="164">
         <f>-IF(COUNTIF($A$6:A122,A122)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A122)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A122),0)</f>
         <v>0</v>
       </c>
@@ -21934,7 +21931,7 @@
         <f t="shared" si="12"/>
         <v>-4466720.46</v>
       </c>
-      <c r="G123" s="167">
+      <c r="G123" s="164">
         <f>-IF(COUNTIF($A$6:A123,A123)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A123)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A123),0)</f>
         <v>0</v>
       </c>
@@ -21964,7 +21961,7 @@
         <f t="shared" si="12"/>
         <v>-4150000</v>
       </c>
-      <c r="G124" s="167">
+      <c r="G124" s="164">
         <f>-IF(COUNTIF($A$6:A124,A124)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A124)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A124),0)</f>
         <v>0</v>
       </c>
@@ -21992,7 +21989,7 @@
         <f t="shared" ref="E125" si="13">-D125+C125</f>
         <v>184102954.74000001</v>
       </c>
-      <c r="G125" s="167">
+      <c r="G125" s="164">
         <f>-IF(COUNTIF($A$6:A125,A125)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A125)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A125),0)</f>
         <v>0</v>
       </c>
@@ -22022,7 +22019,7 @@
         <f t="shared" si="12"/>
         <v>-7000000</v>
       </c>
-      <c r="G126" s="167">
+      <c r="G126" s="164">
         <f>-IF(COUNTIF($A$6:A126,A126)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A126)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A126),0)</f>
         <v>0</v>
       </c>
@@ -22049,12 +22046,12 @@
         <f>+C127</f>
         <v>0</v>
       </c>
-      <c r="G127" s="167">
+      <c r="G127" s="164">
         <f>-IF(COUNTIF($A$6:A127,A127)=1,SUMIFS(Ledger!$O$5:$O$94,Ledger!$M$5:$M$94,A127)+SUMIFS(Ledger!$P$5:$P$94,Ledger!$M$5:$M$94,A127),0)</f>
         <v>0</v>
       </c>
       <c r="H127" s="59">
-        <f t="shared" ref="H71:H127" si="15">C127+G127</f>
+        <f t="shared" ref="H127" si="15">C127+G127</f>
         <v>0</v>
       </c>
     </row>
@@ -22067,7 +22064,7 @@
         <v>210714565.04000002</v>
       </c>
       <c r="D129" s="62"/>
-      <c r="G129" s="163">
+      <c r="G129" s="161">
         <f>SUM(G6:G127)</f>
         <v>-48799976.904532284</v>
       </c>
@@ -22113,7 +22110,7 @@
       <c r="A134" t="s">
         <v>463</v>
       </c>
-      <c r="C134" s="164">
+      <c r="C134" s="162">
         <f>XIRR(H6:H126,A6:A126)</f>
         <v>7.3729541897773768E-2</v>
       </c>
@@ -22172,7 +22169,7 @@
       <c r="C139" s="58"/>
     </row>
     <row r="140" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="D140" s="165"/>
+      <c r="D140" s="163"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -23255,6 +23252,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="2f45b716-dbbf-4eeb-93ba-8cf34a0ba9d6" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c18dbfbf-249c-4ee0-9565-8e61e153ce87">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010089B309425403A6458BFCEC509EB7BC54" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f4bb991a7404b48da9c8c3b904bb3ee">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c18dbfbf-249c-4ee0-9565-8e61e153ce87" xmlns:ns3="2f45b716-dbbf-4eeb-93ba-8cf34a0ba9d6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b61565140b4f6e65289a02eb0f19df99" ns2:_="" ns3:_="">
     <xsd:import namespace="c18dbfbf-249c-4ee0-9565-8e61e153ce87"/>
@@ -23495,17 +23503,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="2f45b716-dbbf-4eeb-93ba-8cf34a0ba9d6" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c18dbfbf-249c-4ee0-9565-8e61e153ce87">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C37CD5A-F832-464E-A9CA-6C75D915F0E3}">
   <ds:schemaRefs>
@@ -23515,6 +23512,23 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1820BF9-F79E-47E9-ABEA-C397D0C9E6E4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c18dbfbf-249c-4ee0-9565-8e61e153ce87"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="2f45b716-dbbf-4eeb-93ba-8cf34a0ba9d6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{01399F26-1612-4A78-A8B5-201010F89563}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -23531,21 +23545,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1820BF9-F79E-47E9-ABEA-C397D0C9E6E4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="c18dbfbf-249c-4ee0-9565-8e61e153ce87"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="2f45b716-dbbf-4eeb-93ba-8cf34a0ba9d6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Fix exact column mappings: Col 12 MOIC, Col 13 IRR, Col 10 NAV
</commit_message>
<xml_diff>
--- a/KAHF_Consolidated_Fund_Model  Updated.xlsx
+++ b/KAHF_Consolidated_Fund_Model  Updated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://konigsteincapital-my.sharepoint.com/personal/wayne_konigsteincapital_com/Documents/Project Images/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1500" documentId="8_{9150A69C-E6E4-4446-B489-F85005C0890C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{379ACD62-8115-43E3-9302-EB0857A0BBD6}"/>
+  <xr:revisionPtr revIDLastSave="1506" documentId="8_{9150A69C-E6E4-4446-B489-F85005C0890C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D86DDF91-5976-4EB4-B63B-DC59A3785ADE}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-4200" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2368,11 +2368,11 @@
     <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="176" fontId="41" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="41" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="39" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -6237,10 +6237,10 @@
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="O30" s="172" t="s">
+      <c r="O30" s="171" t="s">
         <v>321</v>
       </c>
-      <c r="P30" s="172"/>
+      <c r="P30" s="171"/>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.3">
       <c r="P31" t="s">
@@ -12177,12 +12177,12 @@
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="M3" s="173" t="s">
+      <c r="M3" s="172" t="s">
         <v>456</v>
       </c>
-      <c r="N3" s="173"/>
-      <c r="O3" s="173"/>
-      <c r="P3" s="173"/>
+      <c r="N3" s="172"/>
+      <c r="O3" s="172"/>
+      <c r="P3" s="172"/>
     </row>
     <row r="4" spans="1:16" ht="42" x14ac:dyDescent="0.3">
       <c r="A4" s="35" t="s">
@@ -17749,9 +17749,9 @@
         <v>183</v>
       </c>
       <c r="B4" s="47"/>
-      <c r="C4" s="171"/>
-      <c r="D4" s="171"/>
-      <c r="E4" s="171"/>
+      <c r="C4" s="173"/>
+      <c r="D4" s="173"/>
+      <c r="E4" s="173"/>
       <c r="J4" s="166">
         <f>IF(M3&gt;0,L3,J3)</f>
         <v>0</v>
@@ -23243,26 +23243,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="2f45b716-dbbf-4eeb-93ba-8cf34a0ba9d6" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c18dbfbf-249c-4ee0-9565-8e61e153ce87">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010089B309425403A6458BFCEC509EB7BC54" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f4bb991a7404b48da9c8c3b904bb3ee">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c18dbfbf-249c-4ee0-9565-8e61e153ce87" xmlns:ns3="2f45b716-dbbf-4eeb-93ba-8cf34a0ba9d6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b61565140b4f6e65289a02eb0f19df99" ns2:_="" ns3:_="">
     <xsd:import namespace="c18dbfbf-249c-4ee0-9565-8e61e153ce87"/>
@@ -23503,10 +23483,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="2f45b716-dbbf-4eeb-93ba-8cf34a0ba9d6" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c18dbfbf-249c-4ee0-9565-8e61e153ce87">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C37CD5A-F832-464E-A9CA-6C75D915F0E3}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{01399F26-1612-4A78-A8B5-201010F89563}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c18dbfbf-249c-4ee0-9565-8e61e153ce87"/>
+    <ds:schemaRef ds:uri="2f45b716-dbbf-4eeb-93ba-8cf34a0ba9d6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -23529,20 +23540,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{01399F26-1612-4A78-A8B5-201010F89563}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C37CD5A-F832-464E-A9CA-6C75D915F0E3}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="c18dbfbf-249c-4ee0-9565-8e61e153ce87"/>
-    <ds:schemaRef ds:uri="2f45b716-dbbf-4eeb-93ba-8cf34a0ba9d6"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update fund model figures
</commit_message>
<xml_diff>
--- a/KAHF_Consolidated_Fund_Model  Updated.xlsx
+++ b/KAHF_Consolidated_Fund_Model  Updated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://konigsteincapital-my.sharepoint.com/personal/wayne_konigsteincapital_com/Documents/Project Images/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1506" documentId="8_{9150A69C-E6E4-4446-B489-F85005C0890C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D86DDF91-5976-4EB4-B63B-DC59A3785ADE}"/>
+  <xr:revisionPtr revIDLastSave="1507" documentId="8_{9150A69C-E6E4-4446-B489-F85005C0890C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{995DFD0C-5FDE-4980-850D-FFFB8F4CE00F}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-4200" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5492,7 +5492,7 @@
         <v>0.80679453239954835</v>
       </c>
       <c r="M5" s="16">
-        <v>8.7400000000000005E-2</v>
+        <v>0.19750000000000001</v>
       </c>
       <c r="N5" s="17" t="s">
         <v>73</v>
@@ -6155,7 +6155,7 @@
       </c>
       <c r="M19" s="72">
         <f>(M5+M18+M17+M16+M15+M14+M13+M11+M10+M9-M8+M6+M7+M20)/13</f>
-        <v>0.18930769230769234</v>
+        <v>0.1977769230769231</v>
       </c>
       <c r="N19" s="20"/>
     </row>

</xml_diff>